<commit_message>
GZYHTZJY-308 CLONE - 计划类利率型查询
</commit_message>
<xml_diff>
--- a/tams-invest-parent/tams-invest-asset/src/main/resources/tpl/FinPlanProfitAsset.xlsx
+++ b/tams-invest-parent/tams-invest-asset/src/main/resources/tpl/FinPlanProfitAsset.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\ChongQingTouZi\tams\tams-invest-parent\tams-invest-asset\src\main\resources\tpl\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\guangzhoucode\tams\tams-invest-parent\tams-invest-asset\src\main\resources\tpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18276" windowHeight="5916"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18270" windowHeight="5910"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,8 @@
     <t>发行人</t>
   </si>
   <si>
-    <t>母计划</t>
+    <t>托管人</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -164,7 +165,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -199,7 +200,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -409,9 +410,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -431,22 +432,22 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -458,7 +459,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -468,7 +469,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>